<commit_message>
Chose Cherry MX Green Switches for the mute buttons for that good decisive click
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -83,6 +83,40 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/pcf8574rgtr-texas+instruments-666200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k Rotary Poteniometer w/ push switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bourns 39LA-1PB-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/39la-1pb-103-bourns-578549</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cherry MX Green Mechanical Switch Kit</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DMX1A-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">F1NA-1A</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -97,11 +131,12 @@
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -121,6 +156,12 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -167,24 +208,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -311,155 +356,197 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="33.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="7.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="59.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="6.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="7.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="78.8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>5.28</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <f aca="false">D2*C2</f>
         <v>5.28</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>0.74</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <f aca="false">D3*C3</f>
         <v>1.48</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>17.5</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">D4*C4</f>
         <v>70</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>6.17</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">D5*C5</f>
-        <v>61.7</v>
-      </c>
-      <c r="F5" s="3" t="s">
+        <v>37.02</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <f aca="false">D6*C6</f>
         <v>4.5</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>18.89</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <f aca="false">D7*C7</f>
+        <v>37.78</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="2" t="n">
-        <f aca="false">SUM(E2:E7)</f>
-        <v>142.96</v>
+      <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>15.99</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <f aca="false">D8*C8</f>
+        <v>15.99</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="3" t="n">
+        <f aca="false">SUM(E2:E9)</f>
+        <v>172.05</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C10:D10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -467,6 +554,8 @@
     <hyperlink ref="F4" r:id="rId3" display="https://octopart.com/326-adafruit+industries-29717946"/>
     <hyperlink ref="F5" r:id="rId4" display="https://octopart.com/ptl01-15r0-103b1-bourns-77838499"/>
     <hyperlink ref="F6" r:id="rId5" display="https://octopart.com/pcf8574rgtr-texas+instruments-666200"/>
+    <hyperlink ref="F7" r:id="rId6" display="https://octopart.com/39la-1pb-103-bourns-578549"/>
+    <hyperlink ref="F8" r:id="rId7" display="https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Figured out componentes for hardware debouncing and making sure all components have 3D models for when it comes time to make an enclosure
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -97,26 +97,64 @@
     <t xml:space="preserve">Cherry MX Green Mechanical Switch Kit</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DMX1A-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">F1NA-1A</t>
-    </r>
+    <t xml:space="preserve">DMX1A-F1NA-1A</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quad-Schmitt Trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI SN74HCS126DR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/sn74hcs126dr-texas+instruments-110195206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay 0.1uF Polarized Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">293D104X0035A2TE3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/293d104x0035a2te3-vishay-42464905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 1K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6-1879336-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/6-1879336-2-te+connectivity-42430722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 10K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1614881-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1614881-1-te+connectivity-40125137</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onsemi 100V 0.2A Rectifier Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMSD4148T1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/mmsd4148t1g-onsemi-331798</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE COnnectivity 100 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1622828-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1622828-1-te+connectivity-41187673</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -131,7 +169,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -159,11 +197,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -356,7 +389,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
@@ -492,7 +525,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -534,19 +567,145 @@
         <v>26</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <f aca="false">D9*C9</f>
+        <v>0.44</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="5"/>
+      <c r="A10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.41</v>
+      </c>
       <c r="E10" s="3" t="n">
-        <f aca="false">SUM(E2:E9)</f>
-        <v>172.05</v>
+        <f aca="false">D10*C10</f>
+        <v>3.28</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <f aca="false">D11*C11</f>
+        <v>0.8</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <f aca="false">D12*C12</f>
+        <v>1.44</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <f aca="false">D13*C13</f>
+        <v>0.8</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <f aca="false">D14*C14</f>
+        <v>0.6</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="3" t="n">
+        <f aca="false">SUM(E2:E15)</f>
+        <v>179.41</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C16:D16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -556,6 +715,12 @@
     <hyperlink ref="F6" r:id="rId5" display="https://octopart.com/pcf8574rgtr-texas+instruments-666200"/>
     <hyperlink ref="F7" r:id="rId6" display="https://octopart.com/39la-1pb-103-bourns-578549"/>
     <hyperlink ref="F8" r:id="rId7" display="https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1"/>
+    <hyperlink ref="F9" r:id="rId8" display="https://octopart.com/sn74hcs126dr-texas+instruments-110195206"/>
+    <hyperlink ref="F10" r:id="rId9" display="https://octopart.com/293d104x0035a2te3-vishay-42464905"/>
+    <hyperlink ref="F11" r:id="rId10" display="https://octopart.com/6-1879336-2-te+connectivity-42430722"/>
+    <hyperlink ref="F12" r:id="rId11" display="https://octopart.com/1614881-1-te+connectivity-40125137"/>
+    <hyperlink ref="F13" r:id="rId12" display="https://octopart.com/mmsd4148t1g-onsemi-331798"/>
+    <hyperlink ref="F14" r:id="rId13" display="https://octopart.com/1622828-1-te+connectivity-41187673"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
3D File, ESD, and Old File Clean up
* Added the 3D files for the rotary potentiometer with switch.
* Started adding ESD diodes to components the user will touch regularly.
* Removed old files that won't be used.
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -155,6 +155,48 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/1622828-1-te+connectivity-41187673</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 0.1uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCJ188R71H104KA12D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/gcj188r71h104ka12d-murata-20842003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 499 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-3EKF4990V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-3ekf4990v-panasonic-55421795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM USB Choke and ESD Filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECMF02-2AMX6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM ESD Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESDA25P35-1U1M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESDALC6V1-1U2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -169,12 +211,11 @@
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -196,7 +237,12 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -241,7 +287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -259,6 +305,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -389,7 +439,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
@@ -693,19 +743,124 @@
         <v>44</v>
       </c>
     </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <f aca="false">D15*C15</f>
+        <v>1.92</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="5"/>
+      <c r="A16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E16" s="3" t="n">
-        <f aca="false">SUM(E2:E15)</f>
-        <v>179.41</v>
+        <f aca="false">D16*C16</f>
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <f aca="false">D17*C17</f>
+        <v>0.41</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <f aca="false">D18*C18</f>
+        <v>0.37</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <f aca="false">D19*C19</f>
+        <v>4</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="3" t="n">
+        <f aca="false">SUM(E2:E19)</f>
+        <v>186.31</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -721,6 +876,11 @@
     <hyperlink ref="F12" r:id="rId11" display="https://octopart.com/1614881-1-te+connectivity-40125137"/>
     <hyperlink ref="F13" r:id="rId12" display="https://octopart.com/mmsd4148t1g-onsemi-331798"/>
     <hyperlink ref="F14" r:id="rId13" display="https://octopart.com/1622828-1-te+connectivity-41187673"/>
+    <hyperlink ref="F15" r:id="rId14" display="https://octopart.com/gcj188r71h104ka12d-murata-20842003"/>
+    <hyperlink ref="F16" r:id="rId15" display="https://octopart.com/erj-3ekf4990v-panasonic-55421795"/>
+    <hyperlink ref="F17" r:id="rId16" display="https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078"/>
+    <hyperlink ref="F18" r:id="rId17" display="https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699"/>
+    <hyperlink ref="F19" r:id="rId18" display="https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
USB Supporting Hardware, 3D Models, BOM Updates
* Added supporting hardware for the USB C connector
* Ensured all current components have 3D models
* Updated the BOM with components for the USB connector
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -197,6 +197,24 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 5.1K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-3EKF5101V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-3ekf5101v-panasonic-55421801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCT USB C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB4085-GF-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/usb4085-gf-a-global+connector+technology-94773699</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -211,11 +229,12 @@
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -237,12 +256,7 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -287,7 +301,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -305,10 +319,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -439,7 +449,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
@@ -802,7 +812,7 @@
         <f aca="false">D17*C17</f>
         <v>0.41</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="4" t="s">
         <v>53</v>
       </c>
     </row>
@@ -823,7 +833,7 @@
         <f aca="false">D18*C18</f>
         <v>0.37</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="4" t="s">
         <v>56</v>
       </c>
     </row>
@@ -844,23 +854,65 @@
         <f aca="false">D19*C19</f>
         <v>4</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="4" t="s">
         <v>58</v>
       </c>
     </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <f aca="false">D20*C20</f>
+        <v>0.2</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="6"/>
+      <c r="A21" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.88</v>
+      </c>
       <c r="E21" s="3" t="n">
+        <f aca="false">D21*C21</f>
+        <v>0.88</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C23" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="3" t="n">
         <f aca="false">SUM(E2:E19)</f>
         <v>186.31</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C23:D23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -881,6 +933,8 @@
     <hyperlink ref="F17" r:id="rId16" display="https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078"/>
     <hyperlink ref="F18" r:id="rId17" display="https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699"/>
     <hyperlink ref="F19" r:id="rId18" display="https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330"/>
+    <hyperlink ref="F20" r:id="rId19" display="https://octopart.com/erj-3ekf5101v-panasonic-55421801"/>
+    <hyperlink ref="F21" r:id="rId20" display="https://octopart.com/usb4085-gf-a-global+connector+technology-94773699"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Added Footprints and 3D Files
- Added the proper footprint and 3D file for the ESP32
- Added the footprint and 3D file for the USB choke/ESD so the project
  doesn't rely on an external library
- Added the power step down circuit and LED indicators
- Added a user LED for program status
- Made a "Good Enough for Government Work" symbol and footprint for
  the Bourns rotary potentiometer I want to use while I wait for
  SamacSys
- Updated the BOM
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="87">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -215,6 +215,69 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/usb4085-gf-a-global+connector+technology-94773699</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI 5V to 3.3V 5A LDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LMS1585ACS-3.3/NOPB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 10uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM188D71A106MA73D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/grm188d71a106ma73d-murata-26982325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Red LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMS1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlms1300-gs08-vishay-21709201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 200 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-PA3F2000V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-pa3f2000v-panasonic-51302339</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Orange LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMO1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlmo1300-gs08-vishay-21709200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Green LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMTG1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlmtg1300-gs08-vishay-21709202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 10 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRGH0603J10R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/crgh0603j10r-te+connectivity-24382088</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -449,8 +512,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.54"/>
@@ -740,14 +803,14 @@
         <v>43</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.1</v>
       </c>
       <c r="E14" s="3" t="n">
         <f aca="false">D14*C14</f>
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>44</v>
@@ -900,19 +963,166 @@
         <v>64</v>
       </c>
     </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <f aca="false">D22*C22</f>
+        <v>3.57</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="5"/>
+      <c r="A23" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.26</v>
+      </c>
       <c r="E23" s="3" t="n">
+        <f aca="false">D23*C23</f>
+        <v>0.52</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <f aca="false">D24*C24</f>
+        <v>0.21</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <f aca="false">D25*C25</f>
+        <v>0.12</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <f aca="false">D26*C26</f>
+        <v>0.22</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <f aca="false">D27*C27</f>
+        <v>0.34</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <f aca="false">D28*C28</f>
+        <v>0.1</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="3" t="n">
         <f aca="false">SUM(E2:E19)</f>
-        <v>186.31</v>
+        <v>186.41</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C30:D30"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -935,6 +1145,13 @@
     <hyperlink ref="F19" r:id="rId18" display="https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330"/>
     <hyperlink ref="F20" r:id="rId19" display="https://octopart.com/erj-3ekf5101v-panasonic-55421801"/>
     <hyperlink ref="F21" r:id="rId20" display="https://octopart.com/usb4085-gf-a-global+connector+technology-94773699"/>
+    <hyperlink ref="F22" r:id="rId21" display="https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787"/>
+    <hyperlink ref="F23" r:id="rId22" display="https://octopart.com/grm188d71a106ma73d-murata-26982325"/>
+    <hyperlink ref="F24" r:id="rId23" display="https://octopart.com/vlms1300-gs08-vishay-21709201"/>
+    <hyperlink ref="F25" r:id="rId24" display="https://octopart.com/erj-pa3f2000v-panasonic-51302339"/>
+    <hyperlink ref="F26" r:id="rId25" display="https://octopart.com/vlmo1300-gs08-vishay-21709200"/>
+    <hyperlink ref="F27" r:id="rId26" display="https://octopart.com/vlmtg1300-gs08-vishay-21709202"/>
+    <hyperlink ref="F28" r:id="rId27" display="https://octopart.com/crgh0603j10r-te+connectivity-24382088"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Migrated Project Footprints to KiCAD Stable
- I updated the project footprints to be compatable with KiCAD stable
  release.
- I replaced the footprint for the slide potentiometer.
- I corrected the Adafruit display in the BOM sheet since I swapped it
  out a few commits ago.
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -61,10 +61,10 @@
     <t xml:space="preserve">128x64 OLED</t>
   </si>
   <si>
-    <t xml:space="preserve">Adafruit 326</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/326-adafruit+industries-29717946</t>
+    <t xml:space="preserve">Adafruit 938</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/938-adafruit+industries-32979003</t>
   </si>
   <si>
     <t xml:space="preserve">100mm 10k Slide Potentiameter w/ LED</t>
@@ -1127,7 +1127,7 @@
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
     <hyperlink ref="F3" r:id="rId2" display="https://octopart.com/in-pi55qatprpgpbpw-40-inolux-96300409"/>
-    <hyperlink ref="F4" r:id="rId3" display="https://octopart.com/326-adafruit+industries-29717946"/>
+    <hyperlink ref="F4" r:id="rId3" display="https://octopart.com/938-adafruit+industries-32979003"/>
     <hyperlink ref="F5" r:id="rId4" display="https://octopart.com/ptl01-15r0-103b1-bourns-77838499"/>
     <hyperlink ref="F6" r:id="rId5" display="https://octopart.com/pcf8574rgtr-texas+instruments-666200"/>
     <hyperlink ref="F7" r:id="rId6" display="https://octopart.com/39la-1pb-103-bourns-578549"/>

</xml_diff>

<commit_message>
Still dealing with KiCAD Migration issues
- Had to spend way too much time fixing the libraries.
- Adjusted the Adafruit 1.3" OLED footprint 3D model to use a lower
  profile pin headder.
- Added the lower profile pins to the BOM.
- Went through some of the ERC and fixed some issues (most relating to
  the library issues mentioned above).
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="93">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -278,6 +278,24 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/crgh0603j10r-te+connectivity-24382088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preci-Dip Male Connector 1x8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">350-80-108-00-001101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/350-80-108-00-001101-preci-dip-23717904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preci-Dip Female Connector 1x8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">801-87-008-10-012101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/801-87-008-10-012101-preci-dip-23373227</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -512,8 +530,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.54"/>
@@ -1110,19 +1128,61 @@
         <v>85</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <f aca="false">D29*C29</f>
+        <v>4.48</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="5"/>
+      <c r="A30" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1.11</v>
+      </c>
       <c r="E30" s="3" t="n">
+        <f aca="false">D30*C30</f>
+        <v>4.44</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="3" t="n">
         <f aca="false">SUM(E2:E19)</f>
         <v>186.41</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C32:D32"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -1152,6 +1212,8 @@
     <hyperlink ref="F26" r:id="rId25" display="https://octopart.com/vlmo1300-gs08-vishay-21709200"/>
     <hyperlink ref="F27" r:id="rId26" display="https://octopart.com/vlmtg1300-gs08-vishay-21709202"/>
     <hyperlink ref="F28" r:id="rId27" display="https://octopart.com/crgh0603j10r-te+connectivity-24382088"/>
+    <hyperlink ref="F29" r:id="rId28" display="https://octopart.com/350-80-108-00-001101-preci-dip-23717904"/>
+    <hyperlink ref="F30" r:id="rId29" display="https://octopart.com/801-87-008-10-012101-preci-dip-23373227"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Finished Schemtic 🎉      For now...
- Added supporting hardware for the ESP32-S3 (decoupling capacitors and
  reset button)
- Added hardware support for a UART conntection (hoping I won't need to
  use it but you never know)
- Fixed all ERC issues
- Replaced the original 11mm stand offs with 8mm stand offs for the
  Adafruit displays
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="105">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -296,6 +296,42 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/801-87-008-10-012101-preci-dip-23373227</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity SMD Push Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1437566-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1437566-3-te+connectivity-40512141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 22uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM188R61A226ME15D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/grm188r61a226me15d-murata-39203794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 1uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCM188R71E105KA64D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/gcm188r71e105ka64d-murata-18909256</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harwin 8mm Thredded Standoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R30-1000802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/r30-1000802-harwin-792462</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -530,7 +566,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
@@ -779,14 +815,14 @@
         <v>37</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0.18</v>
       </c>
       <c r="E12" s="3" t="n">
         <f aca="false">D12*C12</f>
-        <v>1.44</v>
+        <v>1.62</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>38</v>
@@ -842,14 +878,14 @@
         <v>46</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0.12</v>
       </c>
       <c r="E15" s="3" t="n">
         <f aca="false">D15*C15</f>
-        <v>1.92</v>
+        <v>2.16</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>47</v>
@@ -1073,14 +1109,14 @@
         <v>78</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0.22</v>
       </c>
       <c r="E26" s="3" t="n">
         <f aca="false">D26*C26</f>
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>79</v>
@@ -1170,19 +1206,103 @@
         <v>91</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <f aca="false">D31*C31</f>
+        <v>0.14</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D32" s="5"/>
+      <c r="A32" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0.11</v>
+      </c>
       <c r="E32" s="3" t="n">
+        <f aca="false">D32*C32</f>
+        <v>0.11</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <f aca="false">D33*C33</f>
+        <v>0.19</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <f aca="false">D34*C34</f>
+        <v>4.32</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C36" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="3" t="n">
         <f aca="false">SUM(E2:E19)</f>
-        <v>186.41</v>
+        <v>186.83</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C36:D36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
@@ -1214,6 +1334,10 @@
     <hyperlink ref="F28" r:id="rId27" display="https://octopart.com/crgh0603j10r-te+connectivity-24382088"/>
     <hyperlink ref="F29" r:id="rId28" display="https://octopart.com/350-80-108-00-001101-preci-dip-23717904"/>
     <hyperlink ref="F30" r:id="rId29" display="https://octopart.com/801-87-008-10-012101-preci-dip-23373227"/>
+    <hyperlink ref="F31" r:id="rId30" display="https://octopart.com/1437566-3-te+connectivity-40512141"/>
+    <hyperlink ref="F32" r:id="rId31" display="https://octopart.com/grm188r61a226me15d-murata-39203794"/>
+    <hyperlink ref="F33" r:id="rId32" display="https://octopart.com/gcm188r71e105ka64d-murata-18909256"/>
+    <hyperlink ref="F34" r:id="rId33" display="https://octopart.com/r30-1000802-harwin-792462"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Synced the KiCAD BOM and my handmade BOM
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="102">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -40,6 +40,219 @@
     <t xml:space="preserve">Octopart Link</t>
   </si>
   <si>
+    <t xml:space="preserve">Murata 0.1uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCJ188R71H104KA12D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/gcj188r71h104ka12d-murata-20842003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 1uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCM188R71E105KA64D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/gcm188r71e105ka64d-murata-18909256</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 22uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM188R61A226ME15D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/grm188r61a226me15d-murata-39203794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murata 10uF Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM188D71A106MA73D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/grm188d71a106ma73d-murata-26982325</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay 0.1uF Polarized Capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">293D104X0035A2TE3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/293d104x0035a2te3-vishay-42464905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM ESD Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESDA25P35-1U1M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESDALC6V1-1U2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Red LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMS1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlms1300-gs08-vishay-21709201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGBW LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN-PI55QATPRPGPBPW-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/in-pi55qatprpgpbpw-40-inolux-96300409</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Orange LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMO1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlmo1300-gs08-vishay-21709200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onsemi 100V 0.2A Rectifier Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMSD4148T1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/mmsd4148t1g-onsemi-331798</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay Green LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLMTG1300-GS08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/vlmtg1300-gs08-vishay-21709202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCT USB C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB4085-GF-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/usb4085-gf-a-global+connector+technology-94773699</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100mm 10k Slide Potentiameter w/ LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bourns PTL01-15R0-103B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/ptl01-15r0-103b1-bourns-77838499</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 10K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1614881-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1614881-1-te+connectivity-40125137</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 5.1K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-3EKF5101V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-3ekf5101v-panasonic-55421801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 200 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-PA3F2000V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-pa3f2000v-panasonic-51302339</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic 499 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERJ-3EKF4990V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/erj-3ekf4990v-panasonic-55421795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 100 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1622828-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1622828-1-te+connectivity-41187673</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 1K Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6-1879336-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/6-1879336-2-te+connectivity-42430722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity 10 Ohm Resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRGH0603J10R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/crgh0603j10r-te+connectivity-24382088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE Connectivity SMD Push Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1437566-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/1437566-3-te+connectivity-40512141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cherry MX Green Mechanical Switch Kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMX1A-F1NA-1A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM USB Choke and ESD Filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECMF02-2AMX6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078</t>
+  </si>
+  <si>
     <t xml:space="preserve">ESP32-S3</t>
   </si>
   <si>
@@ -49,13 +262,31 @@
     <t xml:space="preserve">https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335</t>
   </si>
   <si>
-    <t xml:space="preserve">ARGBW LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN-PI55QATPRPGPBPW-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/in-pi55qatprpgpbpw-40-inolux-96300409</t>
+    <t xml:space="preserve">TI 5V to 3.3V 5A LDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LMS1585ACS-3.3/NOPB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k Rotary Poteniometer w/ push switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bourns 39LA-1PB-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/39la-1pb-103-bourns-578549</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quad-Schmitt Trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI SN74HCS126DR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/sn74hcs126dr-texas+instruments-110195206</t>
   </si>
   <si>
     <t xml:space="preserve">128x64 OLED</t>
@@ -67,219 +298,6 @@
     <t xml:space="preserve">https://octopart.com/938-adafruit+industries-32979003</t>
   </si>
   <si>
-    <t xml:space="preserve">100mm 10k Slide Potentiameter w/ LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bourns PTL01-15R0-103B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/ptl01-15r0-103b1-bourns-77838499</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 GPIO Expander</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TI PCF8574RGTR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/pcf8574rgtr-texas+instruments-666200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10k Rotary Poteniometer w/ push switch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bourns 39LA-1PB-103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/39la-1pb-103-bourns-578549</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cherry MX Green Mechanical Switch Kit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMX1A-F1NA-1A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quad-Schmitt Trigger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TI SN74HCS126DR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/sn74hcs126dr-texas+instruments-110195206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishay 0.1uF Polarized Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">293D104X0035A2TE3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/293d104x0035a2te3-vishay-42464905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE Connectivity 1K Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6-1879336-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/6-1879336-2-te+connectivity-42430722</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE Connectivity 10K Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1614881-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/1614881-1-te+connectivity-40125137</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onsemi 100V 0.2A Rectifier Diode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMSD4148T1G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/mmsd4148t1g-onsemi-331798</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE COnnectivity 100 Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1622828-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/1622828-1-te+connectivity-41187673</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murata 0.1uF Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GCJ188R71H104KA12D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/gcj188r71h104ka12d-murata-20842003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panasonic 499 Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERJ-3EKF4990V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/erj-3ekf4990v-panasonic-55421795</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM USB Choke and ESD Filter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECMF02-2AMX6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM ESD Diode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESDA25P35-1U1M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESDALC6V1-1U2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panasonic 5.1K Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERJ-3EKF5101V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/erj-3ekf5101v-panasonic-55421801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GCT USB C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB4085-GF-A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/usb4085-gf-a-global+connector+technology-94773699</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TI 5V to 3.3V 5A LDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LMS1585ACS-3.3/NOPB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murata 10uF Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRM188D71A106MA73D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/grm188d71a106ma73d-murata-26982325</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishay Red LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VLMS1300-GS08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/vlms1300-gs08-vishay-21709201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panasonic 200 Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERJ-PA3F2000V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/erj-pa3f2000v-panasonic-51302339</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishay Orange LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VLMO1300-GS08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/vlmo1300-gs08-vishay-21709200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vishay Green LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VLMTG1300-GS08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/vlmtg1300-gs08-vishay-21709202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE Connectivity 10 Ohm Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRGH0603J10R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/crgh0603j10r-te+connectivity-24382088</t>
-  </si>
-  <si>
     <t xml:space="preserve">Preci-Dip Male Connector 1x8</t>
   </si>
   <si>
@@ -296,33 +314,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/801-87-008-10-012101-preci-dip-23373227</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE Connectivity SMD Push Switch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1437566-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/1437566-3-te+connectivity-40512141</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murata 22uF Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRM188R61A226ME15D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/grm188r61a226me15d-murata-39203794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murata 1uF Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GCM188R71E105KA64D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://octopart.com/gcm188r71e105ka64d-murata-18909256</t>
   </si>
   <si>
     <t xml:space="preserve">Harwin 8mm Thredded Standoff</t>
@@ -418,7 +409,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -432,6 +423,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -566,8 +561,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.54"/>
@@ -578,22 +573,22 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -605,16 +600,16 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5.28</v>
+        <v>0.12</v>
       </c>
       <c r="E2" s="3" t="n">
         <f aca="false">D2*C2</f>
-        <v>5.28</v>
-      </c>
-      <c r="F2" s="4" t="s">
+        <v>2.16</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -626,58 +621,58 @@
         <v>10</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.74</v>
+        <v>0.19</v>
       </c>
       <c r="E3" s="3" t="n">
         <f aca="false">D3*C3</f>
-        <v>1.48</v>
-      </c>
-      <c r="F3" s="4" t="s">
+        <v>0.19</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>17.5</v>
+        <v>0.11</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">D4*C4</f>
-        <v>70</v>
-      </c>
-      <c r="F4" s="4" t="s">
+        <v>0.11</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>6.17</v>
+        <v>0.26</v>
       </c>
       <c r="E5" s="3" t="n">
         <f aca="false">D5*C5</f>
-        <v>37.02</v>
-      </c>
-      <c r="F5" s="4" t="s">
+        <v>0.52</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -689,289 +684,289 @@
         <v>19</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.5</v>
+        <v>0.41</v>
       </c>
       <c r="E6" s="3" t="n">
         <f aca="false">D6*C6</f>
-        <v>4.5</v>
-      </c>
-      <c r="F6" s="4" t="s">
+        <v>6.56</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>18.89</v>
+        <v>0.37</v>
       </c>
       <c r="E7" s="3" t="n">
         <f aca="false">D7*C7</f>
-        <v>37.78</v>
-      </c>
-      <c r="F7" s="4" t="s">
+        <v>0.37</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="C8" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>15.99</v>
+        <v>0.25</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">D8*C8</f>
-        <v>15.99</v>
-      </c>
-      <c r="F8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="E9" s="3" t="n">
         <f aca="false">D9*C9</f>
-        <v>0.44</v>
-      </c>
-      <c r="F9" s="4" t="s">
+        <v>0.21</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="C10" s="2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.41</v>
+        <v>0.74</v>
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">D10*C10</f>
-        <v>3.28</v>
-      </c>
-      <c r="F10" s="4" t="s">
+        <v>10.36</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C11" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="E11" s="3" t="n">
         <f aca="false">D11*C11</f>
-        <v>0.8</v>
-      </c>
-      <c r="F11" s="4" t="s">
+        <v>0.44</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="C12" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="E12" s="3" t="n">
         <f aca="false">D12*C12</f>
-        <v>1.62</v>
-      </c>
-      <c r="F12" s="4" t="s">
+        <v>0.8</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="C13" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.1</v>
+        <v>0.34</v>
       </c>
       <c r="E13" s="3" t="n">
         <f aca="false">D13*C13</f>
-        <v>0.8</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>41</v>
+        <v>0.34</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="C14" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.1</v>
+        <v>0.88</v>
       </c>
       <c r="E14" s="3" t="n">
         <f aca="false">D14*C14</f>
-        <v>0.7</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>44</v>
+        <v>0.88</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="C15" s="2" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.12</v>
+        <v>6.17</v>
       </c>
       <c r="E15" s="3" t="n">
         <f aca="false">D15*C15</f>
-        <v>2.16</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>47</v>
+        <v>37.02</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="C16" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="E16" s="3" t="n">
         <f aca="false">D16*C16</f>
-        <v>0.2</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>50</v>
+        <v>1.62</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.41</v>
+        <v>0.1</v>
       </c>
       <c r="E17" s="3" t="n">
         <f aca="false">D17*C17</f>
-        <v>0.41</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>53</v>
+        <v>0.2</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.37</v>
+        <v>0.12</v>
       </c>
       <c r="E18" s="3" t="n">
         <f aca="false">D18*C18</f>
-        <v>0.37</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>56</v>
+        <v>0.12</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="E19" s="3" t="n">
         <f aca="false">D19*C19</f>
-        <v>4</v>
-      </c>
-      <c r="F19" s="4" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -983,16 +978,16 @@
         <v>60</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0.1</v>
       </c>
       <c r="E20" s="3" t="n">
         <f aca="false">D20*C20</f>
-        <v>0.2</v>
-      </c>
-      <c r="F20" s="4" t="s">
+        <v>0.8</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1004,16 +999,16 @@
         <v>63</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.88</v>
+        <v>0.1</v>
       </c>
       <c r="E21" s="3" t="n">
         <f aca="false">D21*C21</f>
-        <v>0.88</v>
-      </c>
-      <c r="F21" s="4" t="s">
+        <v>0.8</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1028,13 +1023,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>3.57</v>
+        <v>0.1</v>
       </c>
       <c r="E22" s="3" t="n">
         <f aca="false">D22*C22</f>
-        <v>3.57</v>
-      </c>
-      <c r="F22" s="4" t="s">
+        <v>0.1</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1046,16 +1041,16 @@
         <v>69</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.26</v>
+        <v>0.14</v>
       </c>
       <c r="E23" s="3" t="n">
         <f aca="false">D23*C23</f>
-        <v>0.52</v>
-      </c>
-      <c r="F23" s="4" t="s">
+        <v>0.14</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1070,13 +1065,13 @@
         <v>1</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.21</v>
+        <v>15.99</v>
       </c>
       <c r="E24" s="3" t="n">
         <f aca="false">D24*C24</f>
-        <v>0.21</v>
-      </c>
-      <c r="F24" s="4" t="s">
+        <v>15.99</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1091,13 +1086,13 @@
         <v>1</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.12</v>
+        <v>0.41</v>
       </c>
       <c r="E25" s="3" t="n">
         <f aca="false">D25*C25</f>
-        <v>0.12</v>
-      </c>
-      <c r="F25" s="4" t="s">
+        <v>0.41</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1109,16 +1104,16 @@
         <v>78</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.22</v>
+        <v>5.28</v>
       </c>
       <c r="E26" s="3" t="n">
         <f aca="false">D26*C26</f>
-        <v>0.44</v>
-      </c>
-      <c r="F26" s="4" t="s">
+        <v>5.28</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1133,13 +1128,13 @@
         <v>1</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.34</v>
+        <v>3.57</v>
       </c>
       <c r="E27" s="3" t="n">
         <f aca="false">D27*C27</f>
-        <v>0.34</v>
-      </c>
-      <c r="F27" s="4" t="s">
+        <v>3.57</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1151,16 +1146,16 @@
         <v>84</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.1</v>
+        <v>18.89</v>
       </c>
       <c r="E28" s="3" t="n">
         <f aca="false">D28*C28</f>
-        <v>0.1</v>
-      </c>
-      <c r="F28" s="4" t="s">
+        <v>37.78</v>
+      </c>
+      <c r="F28" s="5" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1172,16 +1167,16 @@
         <v>87</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1.12</v>
+        <v>0.22</v>
       </c>
       <c r="E29" s="3" t="n">
         <f aca="false">D29*C29</f>
-        <v>4.48</v>
-      </c>
-      <c r="F29" s="4" t="s">
+        <v>0.44</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1196,13 +1191,13 @@
         <v>4</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1.11</v>
+        <v>17.5</v>
       </c>
       <c r="E30" s="3" t="n">
         <f aca="false">D30*C30</f>
-        <v>4.44</v>
-      </c>
-      <c r="F30" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="5" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1214,16 +1209,16 @@
         <v>93</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.14</v>
+        <v>1.12</v>
       </c>
       <c r="E31" s="3" t="n">
         <f aca="false">D31*C31</f>
-        <v>0.14</v>
-      </c>
-      <c r="F31" s="4" t="s">
+        <v>5.6</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1235,16 +1230,16 @@
         <v>96</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.11</v>
+        <v>1.11</v>
       </c>
       <c r="E32" s="3" t="n">
         <f aca="false">D32*C32</f>
-        <v>0.11</v>
-      </c>
-      <c r="F32" s="4" t="s">
+        <v>4.44</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1256,88 +1251,66 @@
         <v>99</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.19</v>
+        <v>0.27</v>
       </c>
       <c r="E33" s="3" t="n">
         <f aca="false">D33*C33</f>
-        <v>0.19</v>
-      </c>
-      <c r="F33" s="4" t="s">
+        <v>4.32</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C35" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <f aca="false">D34*C34</f>
-        <v>4.32</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="3" t="n">
-        <f aca="false">SUM(E2:E19)</f>
-        <v>186.83</v>
+      <c r="D35" s="6"/>
+      <c r="E35" s="3" t="n">
+        <f aca="false">SUM(E2:E33)</f>
+        <v>215.77</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C35:D35"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
-    <hyperlink ref="F3" r:id="rId2" display="https://octopart.com/in-pi55qatprpgpbpw-40-inolux-96300409"/>
-    <hyperlink ref="F4" r:id="rId3" display="https://octopart.com/938-adafruit+industries-32979003"/>
-    <hyperlink ref="F5" r:id="rId4" display="https://octopart.com/ptl01-15r0-103b1-bourns-77838499"/>
-    <hyperlink ref="F6" r:id="rId5" display="https://octopart.com/pcf8574rgtr-texas+instruments-666200"/>
-    <hyperlink ref="F7" r:id="rId6" display="https://octopart.com/39la-1pb-103-bourns-578549"/>
-    <hyperlink ref="F8" r:id="rId7" display="https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1"/>
-    <hyperlink ref="F9" r:id="rId8" display="https://octopart.com/sn74hcs126dr-texas+instruments-110195206"/>
-    <hyperlink ref="F10" r:id="rId9" display="https://octopart.com/293d104x0035a2te3-vishay-42464905"/>
-    <hyperlink ref="F11" r:id="rId10" display="https://octopart.com/6-1879336-2-te+connectivity-42430722"/>
-    <hyperlink ref="F12" r:id="rId11" display="https://octopart.com/1614881-1-te+connectivity-40125137"/>
-    <hyperlink ref="F13" r:id="rId12" display="https://octopart.com/mmsd4148t1g-onsemi-331798"/>
-    <hyperlink ref="F14" r:id="rId13" display="https://octopart.com/1622828-1-te+connectivity-41187673"/>
-    <hyperlink ref="F15" r:id="rId14" display="https://octopart.com/gcj188r71h104ka12d-murata-20842003"/>
-    <hyperlink ref="F16" r:id="rId15" display="https://octopart.com/erj-3ekf4990v-panasonic-55421795"/>
-    <hyperlink ref="F17" r:id="rId16" display="https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078"/>
-    <hyperlink ref="F18" r:id="rId17" display="https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699"/>
-    <hyperlink ref="F19" r:id="rId18" display="https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330"/>
-    <hyperlink ref="F20" r:id="rId19" display="https://octopart.com/erj-3ekf5101v-panasonic-55421801"/>
-    <hyperlink ref="F21" r:id="rId20" display="https://octopart.com/usb4085-gf-a-global+connector+technology-94773699"/>
-    <hyperlink ref="F22" r:id="rId21" display="https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787"/>
-    <hyperlink ref="F23" r:id="rId22" display="https://octopart.com/grm188d71a106ma73d-murata-26982325"/>
-    <hyperlink ref="F24" r:id="rId23" display="https://octopart.com/vlms1300-gs08-vishay-21709201"/>
-    <hyperlink ref="F25" r:id="rId24" display="https://octopart.com/erj-pa3f2000v-panasonic-51302339"/>
-    <hyperlink ref="F26" r:id="rId25" display="https://octopart.com/vlmo1300-gs08-vishay-21709200"/>
-    <hyperlink ref="F27" r:id="rId26" display="https://octopart.com/vlmtg1300-gs08-vishay-21709202"/>
-    <hyperlink ref="F28" r:id="rId27" display="https://octopart.com/crgh0603j10r-te+connectivity-24382088"/>
-    <hyperlink ref="F29" r:id="rId28" display="https://octopart.com/350-80-108-00-001101-preci-dip-23717904"/>
-    <hyperlink ref="F30" r:id="rId29" display="https://octopart.com/801-87-008-10-012101-preci-dip-23373227"/>
-    <hyperlink ref="F31" r:id="rId30" display="https://octopart.com/1437566-3-te+connectivity-40512141"/>
-    <hyperlink ref="F32" r:id="rId31" display="https://octopart.com/grm188r61a226me15d-murata-39203794"/>
-    <hyperlink ref="F33" r:id="rId32" display="https://octopart.com/gcm188r71e105ka64d-murata-18909256"/>
-    <hyperlink ref="F34" r:id="rId33" display="https://octopart.com/r30-1000802-harwin-792462"/>
+    <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/gcj188r71h104ka12d-murata-20842003"/>
+    <hyperlink ref="F3" r:id="rId2" display="https://octopart.com/gcm188r71e105ka64d-murata-18909256"/>
+    <hyperlink ref="F4" r:id="rId3" display="https://octopart.com/grm188r61a226me15d-murata-39203794"/>
+    <hyperlink ref="F5" r:id="rId4" display="https://octopart.com/grm188d71a106ma73d-murata-26982325"/>
+    <hyperlink ref="F6" r:id="rId5" display="https://octopart.com/293d104x0035a2te3-vishay-42464905"/>
+    <hyperlink ref="F7" r:id="rId6" display="https://octopart.com/esda25p35-1u1m-stmicroelectronics-75302699"/>
+    <hyperlink ref="F8" r:id="rId7" display="https://octopart.com/esdalc6v1-1u2-stmicroelectronics-11912330"/>
+    <hyperlink ref="F9" r:id="rId8" display="https://octopart.com/vlms1300-gs08-vishay-21709201"/>
+    <hyperlink ref="F10" r:id="rId9" display="https://octopart.com/in-pi55qatprpgpbpw-40-inolux-96300409"/>
+    <hyperlink ref="F11" r:id="rId10" display="https://octopart.com/vlmo1300-gs08-vishay-21709200"/>
+    <hyperlink ref="F12" r:id="rId11" display="https://octopart.com/mmsd4148t1g-onsemi-331798"/>
+    <hyperlink ref="F13" r:id="rId12" display="https://octopart.com/vlmtg1300-gs08-vishay-21709202"/>
+    <hyperlink ref="F14" r:id="rId13" display="https://octopart.com/usb4085-gf-a-global+connector+technology-94773699"/>
+    <hyperlink ref="F15" r:id="rId14" display="https://octopart.com/ptl01-15r0-103b1-bourns-77838499"/>
+    <hyperlink ref="F16" r:id="rId15" display="https://octopart.com/1614881-1-te+connectivity-40125137"/>
+    <hyperlink ref="F17" r:id="rId16" display="https://octopart.com/erj-3ekf5101v-panasonic-55421801"/>
+    <hyperlink ref="F18" r:id="rId17" display="https://octopart.com/erj-pa3f2000v-panasonic-51302339"/>
+    <hyperlink ref="F19" r:id="rId18" display="https://octopart.com/erj-3ekf4990v-panasonic-55421795"/>
+    <hyperlink ref="F20" r:id="rId19" display="https://octopart.com/1622828-1-te+connectivity-41187673"/>
+    <hyperlink ref="F21" r:id="rId20" display="https://octopart.com/6-1879336-2-te+connectivity-42430722"/>
+    <hyperlink ref="F22" r:id="rId21" display="https://octopart.com/crgh0603j10r-te+connectivity-24382088"/>
+    <hyperlink ref="F23" r:id="rId22" display="https://octopart.com/1437566-3-te+connectivity-40512141"/>
+    <hyperlink ref="F24" r:id="rId23" display="https://www.amazon.com/Cherry-Switch-Mechanical-Keyboard-Switches/dp/B0CXTP79HR?th=1"/>
+    <hyperlink ref="F25" r:id="rId24" display="https://octopart.com/ecmf02-2amx6-stmicroelectronics-44353078"/>
+    <hyperlink ref="F26" r:id="rId25" display="https://octopart.com/esp32-s3-mini-1u-n8-espressif+systems-129194335"/>
+    <hyperlink ref="F27" r:id="rId26" display="https://octopart.com/lms1585acs-3.3%2Fnopb-texas+instruments-24815787"/>
+    <hyperlink ref="F28" r:id="rId27" display="https://octopart.com/39la-1pb-103-bourns-578549"/>
+    <hyperlink ref="F29" r:id="rId28" display="https://octopart.com/sn74hcs126dr-texas+instruments-110195206"/>
+    <hyperlink ref="F30" r:id="rId29" display="https://octopart.com/938-adafruit+industries-32979003"/>
+    <hyperlink ref="F31" r:id="rId30" display="https://octopart.com/350-80-108-00-001101-preci-dip-23717904"/>
+    <hyperlink ref="F32" r:id="rId31" display="https://octopart.com/801-87-008-10-012101-preci-dip-23373227"/>
+    <hyperlink ref="F33" r:id="rId32" display="https://octopart.com/r30-1000802-harwin-792462"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Started PCB Layout Added Mounting Holes and Knobs
- Started doing PCB layout. I have an idea of large component placement
  and therefore overall board size but still working out finalizing
  them.
- Added platted mounting holes to the board mostly for support since
  most of this board is user interfaces I expect there to be a good
  amount of force applied to the sliders, buttons, and knobs.
- Found some metal knobs for the rotary potentiometers and added them to
  the custom BOM.
</commit_message>
<xml_diff>
--- a/Hardware/BrainstormingPartsList.xlsx
+++ b/Hardware/BrainstormingPartsList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="105">
   <si>
     <t xml:space="preserve">Part Name</t>
   </si>
@@ -323,6 +323,15 @@
   </si>
   <si>
     <t xml:space="preserve">https://octopart.com/r30-1000802-harwin-792462</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kilo International Metal Knob</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OEJL-90-4-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://octopart.com/oejl-90-4-6-kilo+international-573308</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -561,7 +570,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.86"/>
@@ -1264,19 +1273,40 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="6" t="s">
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D35" s="6"/>
-      <c r="E35" s="3" t="n">
-        <f aca="false">SUM(E2:E33)</f>
-        <v>215.77</v>
+      <c r="B34" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <f aca="false">D34*C34</f>
+        <v>24.1</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C36" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="3" t="n">
+        <f aca="false">SUM(E2:E34)</f>
+        <v>239.87</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" display="https://octopart.com/gcj188r71h104ka12d-murata-20842003"/>
@@ -1311,6 +1341,7 @@
     <hyperlink ref="F31" r:id="rId30" display="https://octopart.com/350-80-108-00-001101-preci-dip-23717904"/>
     <hyperlink ref="F32" r:id="rId31" display="https://octopart.com/801-87-008-10-012101-preci-dip-23373227"/>
     <hyperlink ref="F33" r:id="rId32" display="https://octopart.com/r30-1000802-harwin-792462"/>
+    <hyperlink ref="F34" r:id="rId33" display="https://octopart.com/oejl-90-4-6-kilo+international-573308"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>